<commit_message>
B16: record hand-verified claims in checked_by
Re-checked 18 claims by hand (P1-01, P2-03, P3-01, P3-07, P3-08,
P5-02, P7-01, P9-01, D1-05, D1-09, D1-14, D1-18, D1-22, Part 3
P3-01, P3-07, P3-08, P3-15, P3-16). D1-22 is now final: Holder is
the N2 Adapter recorded in pattern_evolution.csv. Workbook rebuilt.
</commit_message>
<xml_diff>
--- a/B16/B16_dataset.xlsx
+++ b/B16/B16_dataset.xlsx
@@ -1365,7 +1365,7 @@
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1436,7 +1436,11 @@
           <t>reproduced on my Mac with Java 25 / Python 3.14 / Node 26 / Apple clang 21: 30/30 exit 0; the web run used older versions (Java 21; Python 3.13; Node 22; clang 18)</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr"/>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -1626,7 +1630,11 @@
           <t>difference stated in the READMEs: JUnit catches Throwable and rethrows unrecoverable errors; the snippets catch RuntimeException / Exception / std::exception / any thrown value</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr"/>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -1655,7 +1663,11 @@
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr"/>
-      <c r="G9" s="8" t="inlineStr"/>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -1886,7 +1898,11 @@
           <t>the Java Chain README first said JUnit passes a proceed callback; reworded to Invocation.proceed()</t>
         </is>
       </c>
-      <c r="G16" s="8" t="inlineStr"/>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -1919,7 +1935,11 @@
           <t>lizard 1.24.1 stopped parsing adapter.js inside describe(), at a template literal nested in another one, so max CC was reported as 3; the line was rewritten without nesting (same output, tests 3/3) and lizard then saw every function: max CC 9, matching a manual count. Line counts of all 85 production files agree with an independent count within 10%.</t>
         </is>
       </c>
-      <c r="G17" s="8" t="inlineStr"/>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -19191,7 +19211,7 @@
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19262,7 +19282,11 @@
           <t>8 'missing' entries are only wildcards (tagexpression/*.java, condition/*.java, util/*.java) or '.../' abbreviations; all resolve to real files</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr"/>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -19560,7 +19584,11 @@
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr"/>
-      <c r="G12" s="8" t="inlineStr"/>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -19746,7 +19774,11 @@
           <t>110/110 exact</t>
         </is>
       </c>
-      <c r="G18" s="8" t="inlineStr"/>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -19928,7 +19960,11 @@
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr"/>
-      <c r="G24" s="8" t="inlineStr"/>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -19957,7 +19993,11 @@
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr"/>
-      <c r="G25" s="8" t="inlineStr"/>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -20416,7 +20456,11 @@
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr"/>
-      <c r="G40" s="8" t="inlineStr"/>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
@@ -21003,7 +21047,11 @@
           <t>75/75 exact</t>
         </is>
       </c>
-      <c r="G59" s="8" t="inlineStr"/>
+      <c r="G59" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
@@ -21603,7 +21651,11 @@
           <t>100/100 exact</t>
         </is>
       </c>
-      <c r="G79" s="8" t="inlineStr"/>
+      <c r="G79" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
@@ -22375,9 +22427,9 @@
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -22568,7 +22620,11 @@
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr"/>
-      <c r="G6" s="8" t="inlineStr"/>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -22684,7 +22740,11 @@
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr"/>
-      <c r="G10" s="8" t="inlineStr"/>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -22837,7 +22897,11 @@
           <t>launcherDiscoveryFinished still runs (finally), then the exception escapes Launcher.discover</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr"/>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -22961,7 +23025,11 @@
           <t>in the sketch Mode is only tested in a ternary inside apply(); no behaviour is selected polymorphically, so it is a flag, not a Strategy. Not counted as a new pattern</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr"/>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -23085,15 +23153,19 @@
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>incorrect (proposed)</t>
+          <t>incorrect</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>Holder converts ResourceFactory.destroy(T) into the AutoCloseable/CloseableResource close() that the store close action calls: an object Adapter. Proposed as newly introduced together with the ResourceFactory Strategy (ConcreteStrategy supplied by users; absent from production code); final decision pending in patterns_evolution.csv</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="inlineStr"/>
+          <t>Holder converts ResourceFactory.destroy(T) into the AutoCloseable/CloseableResource close() that the store close action calls: an object Adapter. Counted as newly introduced together with the ResourceFactory Strategy (ConcreteStrategy supplied by users; absent from production code); recorded as N1 Strategy and N2 Adapter (newly_introduced) in Part2/pattern_evolution.csv</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Gautham Mohanraj</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">

</xml_diff>

<commit_message>
B16: update prompt authorship notes in llm.csv
</commit_message>
<xml_diff>
--- a/B16/B16_dataset.xlsx
+++ b/B16/B16_dataset.xlsx
@@ -18508,7 +18508,7 @@
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>correct: all 157 full paths and 262 short file names exist at the commit; 6 behavioural claims spot-checked in source and correct (P1-01..P1-08). Prompt written by me, adapted from a suggestion by Claude.</t>
+          <t>correct: all 157 full paths and 262 short file names exist at the commit; 6 behavioural claims spot-checked in source and correct (P1-01..P1-08). Prompt written by me.</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
@@ -18582,7 +18582,7 @@
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>partially correct: 110/110 cited lines exact; all 5 verdicts supported by source; 2 judgement issues (P3-11 inconsistent Composite rule, P3-12 Strategy/Composite overlap) decided by me. Prompt written by me, adapted from a suggestion by Claude.</t>
+          <t>partially correct: 110/110 cited lines exact; all 5 verdicts supported by source; 2 judgement issues (P3-11 inconsistent Composite rule, P3-12 Strategy/Composite overlap) decided by me. Prompt written by me.</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
@@ -18619,7 +18619,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>partially correct: 6 of 7 checked claims correct; step 7 is wrong - for a @Disabled method the test instance IS created because prepare() runs before shouldBeSkipped() (NodeTestTask.java:109-114, TestMethodTestDescriptor.java:127). Prompt written by me, adapted from a suggestion by Claude.</t>
+          <t>partially correct: 6 of 7 checked claims correct; step 7 is wrong - for a @Disabled method the test instance IS created because prepare() runs before shouldBeSkipped() (NodeTestTask.java:109-114, TestMethodTestDescriptor.java:127). Prompt written by me.</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
@@ -18693,7 +18693,7 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>correct: 103/103 cited lines exact; all verdicts supported by source (P5-01..P5-14). Counting decisions (overlaps, reused Composite, listener classes shared with Area C) made by me. Prompt written by me, adapted from a suggestion by Claude.</t>
+          <t>correct: 103/103 cited lines exact; all verdicts supported by source (P5-01..P5-14). Counting decisions (overlaps, reused Composite, listener classes shared with Area C) made by me. Prompt written by me.</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
@@ -18730,7 +18730,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>correct: 6 checked claims correct (P6-01..P6-06); small omissions only (optional MemoryCleanupListener; engine skipped event is also delayed). Prompt written by me, adapted from a suggestion by Claude.</t>
+          <t>correct: 6 checked claims correct (P6-01..P6-06); small omissions only (optional MemoryCleanupListener; engine skipped event is also delayed). Prompt written by me.</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
@@ -18767,7 +18767,7 @@
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>correct: 75/75 cited lines exact; followed the do-not-recount instruction; one weak claim (ListenerRegistry factory as Strategy) recorded as uncertain (P7-07). Prompt written by me, adapted from a suggestion by Claude.</t>
+          <t>correct: 75/75 cited lines exact; followed the do-not-recount instruction; one weak claim (ListenerRegistry factory as Strategy) recorded as uncertain (P7-07). Prompt written by me.</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
@@ -18804,7 +18804,7 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>correct: 21/21 cited lines correct and 7 behavioural claims confirmed (P8-01..P8-08). Prompt written by me, adapted from a suggestion by Claude.</t>
+          <t>correct: 21/21 cited lines correct and 7 behavioural claims confirmed (P8-01..P8-08). Prompt written by me.</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
@@ -18841,7 +18841,7 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>correct: 100/100 cited lines exact; all verdicts supported (P9-01..P9-16); followed the do-not-recount instruction. Prompt written by me, adapted from a suggestion by Claude.</t>
+          <t>correct: 100/100 cited lines exact; all verdicts supported (P9-01..P9-16); followed the do-not-recount instruction. Prompt written by me.</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
@@ -18878,7 +18878,7 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>partially correct: 98/98 implements/extends arrows match source; 1 wrong participant (A2 EngineFilter) removed; model ids remapped to ours and 2 extra diagrams dropped (P10-01..P10-04). Prompt drafted with Claude, used by me.</t>
+          <t>partially correct: 98/98 implements/extends arrows match source; 1 wrong participant (A2 EngineFilter) removed; model ids remapped to ours and 2 extra diagrams dropped (P10-01..P10-04). Prompt written by me.</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
@@ -18915,7 +18915,7 @@
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>partially correct: 18 of 20 numbered steps correct; step 2 (builder does not call the launcher) and step 8 (DefaultLauncher, not the orchestrator, builds the TestPlan) corrected; wrapper gap annotated (P11-01..P11-05). Prompt drafted with Claude, used by me.</t>
+          <t>partially correct: 18 of 20 numbered steps correct; step 2 (builder does not call the launcher) and step 8 (DefaultLauncher, not the orchestrator, builds the TestPlan) corrected; wrapper gap annotated (P11-01..P11-05). Prompt written by me.</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
@@ -18952,7 +18952,7 @@
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>partially correct: 111/112 line references exact (1 off by one), 2 range ends wrong; 14 behavioural claims checked and correct; pattern ids remapped to ours, 2 non-counted patterns noted; the 'new enum Strategy' claim for CH03 rejected; CH02 code sketch does not compile as written the Long Method label for CH03 is not supported by metrics (D1-01..D1-22; D1-21 added during CH01: the deactivate key only works as a system property; D1-22 added during CH02: Holder is an Adapter). Prompt written by me, adapted from a suggestion by Claude.</t>
+          <t>partially correct: 111/112 line references exact (1 off by one), 2 range ends wrong; 14 behavioural claims checked and correct; pattern ids remapped to ours, 2 non-counted patterns noted; the 'new enum Strategy' claim for CH03 rejected; CH02 code sketch does not compile as written the Long Method label for CH03 is not supported by metrics (D1-01..D1-22; D1-21 added during CH01: the deactivate key only works as a system property; D1-22 added during CH02: Holder is an Adapter). Prompt written by me.</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
@@ -19100,7 +19100,7 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>correct, with 1 partial and 1 not confirmable: all 30 commands re-run on my Mac (Java 25, Python 3.14, Node 26, Apple clang 21) exit 0, 8/8 outputs identical, 0 C++ warnings, ASan/UBSan clean, 0 leaks; partial: 'small production code' (Composite parsers CCN 17-24); cannot confirm: '16 extra inputs' (not in the zip) (P3-01..P3-10). Code used unchanged. Prompt written by me, adapted from a suggestion by Claude. Raw output = the zip (all files + the web sandbox RUN-LOG.txt); the chat reply text was not saved.</t>
+          <t>correct, with 1 partial and 1 not confirmable: all 30 commands re-run on my Mac (Java 25, Python 3.14, Node 26, Apple clang 21) exit 0, 8/8 outputs identical, 0 C++ warnings, ASan/UBSan clean, 0 leaks; partial: 'small production code' (Composite parsers CCN 17-24); cannot confirm: '16 extra inputs' (not in the zip) (P3-01..P3-10). Code used unchanged. Prompt written by me. Raw output = the zip (all files + the web sandbox RUN-LOG.txt); the chat reply text was not saved.</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">

</xml_diff>